<commit_message>
:sparkles: adds German version
</commit_message>
<xml_diff>
--- a/data/output/patient_simulator_comparison.xlsx
+++ b/data/output/patient_simulator_comparison.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bernerfachhochschule.sharepoint.com/sites/ti-smaragd/Freigegebene Dokumente/General/09_Paper/24_LREC-COLING/Workshop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/Projects/patient_vignettes/data/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:40009_{D1E8E7CA-8A0B-1B46-AF16-C3274C6CCF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5660B5E9-28FA-CE4B-A479-16412DF2430A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4562B60A-0625-364B-AD36-EC16BEAE6751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="17280" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3560" yWindow="3640" windowWidth="17280" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="output" sheetId="1" r:id="rId1"/>
@@ -613,7 +613,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1116,48 +1116,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20 % - Akzent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40 % - Akzent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60 % - Akzent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Akzent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Akzent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Akzent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Akzent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Akzent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Akzent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Ausgabe" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Berechnung" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Eingabe" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Ergebnis" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Erklärender Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Gut" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Notiz" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Schlecht" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Überschrift" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Überschrift 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Überschrift 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Überschrift 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Überschrift 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Verknüpfte Zelle" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Warnender Text" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Zelle überprüfen" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1490,13 +1490,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="3" width="50.875" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="10.875" style="2"/>
+    <col min="1" max="3" width="50.83203125" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.100000000000001">
+    <row r="1" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1507,28 +1507,28 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
     </row>
-    <row r="4" spans="1:6" ht="17.100000000000001" customHeight="1">
+    <row r="4" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
     </row>
-    <row r="5" spans="1:6" ht="102">
+    <row r="5" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1551,14 +1551,14 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
     </row>
-    <row r="7" spans="1:6" ht="153">
+    <row r="7" spans="1:6" ht="153" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -1569,26 +1569,26 @@
         <v>12</v>
       </c>
       <c r="D7" s="2">
-        <f t="shared" ref="D6:D25" si="1">IF(LEN(TRIM(A7))=0,0,LEN(TRIM(A7))-LEN(SUBSTITUTE(A7," ",""))+1)</f>
+        <f t="shared" ref="D7:D25" si="1">IF(LEN(TRIM(A7))=0,0,LEN(TRIM(A7))-LEN(SUBSTITUTE(A7," ",""))+1)</f>
         <v>65</v>
       </c>
       <c r="E7" s="2">
-        <f t="shared" ref="E6:E25" si="2">IF(LEN(TRIM(B7))=0,0,LEN(TRIM(B7))-LEN(SUBSTITUTE(B7," ",""))+1)</f>
+        <f t="shared" ref="E7:E25" si="2">IF(LEN(TRIM(B7))=0,0,LEN(TRIM(B7))-LEN(SUBSTITUTE(B7," ",""))+1)</f>
         <v>83</v>
       </c>
       <c r="F7" s="2">
-        <f t="shared" ref="F6:F25" si="3">IF(LEN(TRIM(C7))=0,0,LEN(TRIM(C7))-LEN(SUBSTITUTE(C7," ",""))+1)</f>
+        <f t="shared" ref="F7:F25" si="3">IF(LEN(TRIM(C7))=0,0,LEN(TRIM(C7))-LEN(SUBSTITUTE(C7," ",""))+1)</f>
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="17.100000000000001" customHeight="1">
+    <row r="8" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:6" ht="135.94999999999999">
+    <row r="9" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
@@ -1611,14 +1611,14 @@
         <v>76</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="17.100000000000001" customHeight="1">
+    <row r="10" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:6" ht="119.1">
+    <row r="11" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>18</v>
       </c>
@@ -1641,14 +1641,14 @@
         <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="17.100000000000001" customHeight="1">
+    <row r="12" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:6" ht="170.1">
+    <row r="13" spans="1:6" ht="170" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -1671,14 +1671,14 @@
         <v>111</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="17.100000000000001" customHeight="1">
+    <row r="14" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:6" ht="84.95">
+    <row r="15" spans="1:6" ht="85" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>26</v>
       </c>
@@ -1701,14 +1701,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:6" ht="186.95">
+    <row r="17" spans="1:6" ht="187" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
@@ -1731,14 +1731,14 @@
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
-    <row r="19" spans="1:6" ht="186.95">
+    <row r="19" spans="1:6" ht="187" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>34</v>
       </c>
@@ -1761,14 +1761,14 @@
         <v>112</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="17.100000000000001" customHeight="1">
+    <row r="20" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>37</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
     </row>
-    <row r="21" spans="1:6" ht="135.94999999999999">
+    <row r="21" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>38</v>
       </c>
@@ -1791,14 +1791,14 @@
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="17.100000000000001" customHeight="1">
+    <row r="22" spans="1:6" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>41</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
     </row>
-    <row r="23" spans="1:6" ht="135.94999999999999">
+    <row r="23" spans="1:6" ht="136" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
@@ -1821,14 +1821,14 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>45</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
     </row>
-    <row r="25" spans="1:6" ht="68.099999999999994">
+    <row r="25" spans="1:6" ht="68" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>46</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D26" s="2">
         <f>SUM(D5:D25)</f>
         <v>580</v>
@@ -1865,7 +1865,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D27" s="2">
         <f>D26/11</f>
         <v>52.727272727272727</v>
@@ -1879,12 +1879,12 @@
         <v>78.36363636363636</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>50</v>
       </c>
@@ -1910,17 +1910,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aa40c3e9-d5aa-4736-82da-71b46ec0d168">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4458a041-76dd-4c5b-b387-97f12b754d37" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100310EACFF6E12464E8D0D42AAE93AFDBF" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="efa1b9a215fad520ec0fafcad15e96d6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aa40c3e9-d5aa-4736-82da-71b46ec0d168" xmlns:ns3="4458a041-76dd-4c5b-b387-97f12b754d37" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2c4cd5c46f96ec5bf9062b7e2a5bde23" ns2:_="" ns3:_="">
     <xsd:import namespace="aa40c3e9-d5aa-4736-82da-71b46ec0d168"/>
@@ -2155,6 +2144,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aa40c3e9-d5aa-4736-82da-71b46ec0d168">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4458a041-76dd-4c5b-b387-97f12b754d37" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2165,13 +2165,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8D89D58-8AA5-4ACA-B3E7-43B607C409CA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C55F0C39-C182-493F-B7C5-1D86E7D639C1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="aa40c3e9-d5aa-4736-82da-71b46ec0d168"/>
+    <ds:schemaRef ds:uri="4458a041-76dd-4c5b-b387-97f12b754d37"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C55F0C39-C182-493F-B7C5-1D86E7D639C1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8D89D58-8AA5-4ACA-B3E7-43B607C409CA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="aa40c3e9-d5aa-4736-82da-71b46ec0d168"/>
+    <ds:schemaRef ds:uri="4458a041-76dd-4c5b-b387-97f12b754d37"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CF05BB4-8E75-4A8E-8070-ACEC4560653A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CF05BB4-8E75-4A8E-8070-ACEC4560653A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>